<commit_message>
Incorporar modulos Clima y Mapa, y cambios pendientes del directorio
- Nuevos modulos: Clima laboral (css/clima.css, js/clima.js) y Mapa comercial
  (css/mapa.css, js/mapa.js, js/mapa-data.js, js/mapa-geo.js).
- Ajustes en base, ventas, moventas, clientes, pipeline, organigrama y shared.
- Organigrama: nuevas fotos de Lizeth Arevalo y Valeria Rodriguez; se retiran
  las fotos y archivos que ya no se referencian.
- Actualizacion de las fuentes de datos xlsx (produccion, objetivos, pipeline)
  y alta de la Evaluacion de Clima Laboral.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Friopacking_Objetivos_2_3_4_5.xlsx
+++ b/Friopacking_Objetivos_2_3_4_5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vrodriguez\Desktop\Directorio J\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86072B46-B602-4DAD-93AB-4801FB1081DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9F73501-D9AD-4B24-B256-BB9EA1D7D8BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="180">
   <si>
     <t>OBJETIVO 2 — EJECUTAR PROYECTOS CON REFRIGERANTE CO2</t>
   </si>
@@ -592,7 +592,7 @@
     <numFmt numFmtId="165" formatCode="[$$-540A]#,##0.00"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="169" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="168" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="24" x14ac:knownFonts="1">
     <font>
@@ -1073,7 +1073,7 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1236,30 +1236,6 @@
     <xf numFmtId="0" fontId="12" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1319,37 +1295,61 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1630,84 +1630,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
     </row>
     <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
+      <c r="B3" s="86"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="86"/>
+      <c r="E3" s="86"/>
+      <c r="F3" s="86"/>
+      <c r="G3" s="86"/>
+      <c r="H3" s="86"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="85" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
+      <c r="C4" s="85"/>
+      <c r="D4" s="85"/>
+      <c r="E4" s="85"/>
+      <c r="F4" s="85"/>
+      <c r="G4" s="85"/>
+      <c r="H4" s="85"/>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="54" t="s">
+      <c r="B5" s="85" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="54"/>
+      <c r="C5" s="85"/>
+      <c r="D5" s="85"/>
+      <c r="E5" s="85"/>
+      <c r="F5" s="85"/>
+      <c r="G5" s="85"/>
+      <c r="H5" s="85"/>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
+      <c r="C6" s="85"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="85"/>
+      <c r="F6" s="85"/>
+      <c r="G6" s="85"/>
+      <c r="H6" s="85"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="54" t="s">
+      <c r="B7" s="85" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
-      <c r="H7" s="54"/>
+      <c r="C7" s="85"/>
+      <c r="D7" s="85"/>
+      <c r="E7" s="85"/>
+      <c r="F7" s="85"/>
+      <c r="G7" s="85"/>
+      <c r="H7" s="85"/>
     </row>
     <row r="9" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A9" s="42" t="s">
@@ -1939,148 +1939,148 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="79" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="79"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
+      <c r="B3" s="86"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="86"/>
+      <c r="E3" s="86"/>
+      <c r="F3" s="86"/>
+      <c r="G3" s="86"/>
+      <c r="H3" s="86"/>
+      <c r="I3" s="86"/>
     </row>
     <row r="4" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
+      <c r="C4" s="85"/>
+      <c r="D4" s="85"/>
+      <c r="E4" s="85"/>
+      <c r="F4" s="85"/>
+      <c r="G4" s="85"/>
+      <c r="H4" s="85"/>
+      <c r="I4" s="85"/>
     </row>
     <row r="5" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="54" t="s">
+      <c r="B5" s="85" t="s">
         <v>49</v>
       </c>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="54"/>
-      <c r="I5" s="54"/>
+      <c r="C5" s="85"/>
+      <c r="D5" s="85"/>
+      <c r="E5" s="85"/>
+      <c r="F5" s="85"/>
+      <c r="G5" s="85"/>
+      <c r="H5" s="85"/>
+      <c r="I5" s="85"/>
     </row>
     <row r="6" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
-      <c r="I6" s="54"/>
+      <c r="C6" s="85"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="85"/>
+      <c r="F6" s="85"/>
+      <c r="G6" s="85"/>
+      <c r="H6" s="85"/>
+      <c r="I6" s="85"/>
     </row>
     <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="54" t="s">
+      <c r="B7" s="85" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
-      <c r="H7" s="54"/>
-      <c r="I7" s="54"/>
+      <c r="C7" s="85"/>
+      <c r="D7" s="85"/>
+      <c r="E7" s="85"/>
+      <c r="F7" s="85"/>
+      <c r="G7" s="85"/>
+      <c r="H7" s="85"/>
+      <c r="I7" s="85"/>
     </row>
     <row r="8" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="54" t="s">
+      <c r="B8" s="85" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="54"/>
-      <c r="H8" s="54"/>
-      <c r="I8" s="54"/>
+      <c r="C8" s="85"/>
+      <c r="D8" s="85"/>
+      <c r="E8" s="85"/>
+      <c r="F8" s="85"/>
+      <c r="G8" s="85"/>
+      <c r="H8" s="85"/>
+      <c r="I8" s="85"/>
     </row>
     <row r="9" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="54" t="s">
+      <c r="B9" s="85" t="s">
         <v>55</v>
       </c>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
+      <c r="C9" s="85"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="85"/>
+      <c r="F9" s="85"/>
+      <c r="G9" s="85"/>
+      <c r="H9" s="85"/>
+      <c r="I9" s="85"/>
     </row>
     <row r="10" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="54" t="s">
+      <c r="B10" s="85" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="54"/>
-      <c r="D10" s="54"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="54"/>
-      <c r="H10" s="54"/>
-      <c r="I10" s="54"/>
+      <c r="C10" s="85"/>
+      <c r="D10" s="85"/>
+      <c r="E10" s="85"/>
+      <c r="F10" s="85"/>
+      <c r="G10" s="85"/>
+      <c r="H10" s="85"/>
+      <c r="I10" s="85"/>
     </row>
     <row r="12" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="59" t="s">
+      <c r="A12" s="80" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="59"/>
-      <c r="C12" s="59"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="59"/>
-      <c r="F12" s="59"/>
-      <c r="G12" s="59"/>
-      <c r="H12" s="59"/>
-      <c r="I12" s="59"/>
+      <c r="B12" s="80"/>
+      <c r="C12" s="80"/>
+      <c r="D12" s="80"/>
+      <c r="E12" s="80"/>
+      <c r="F12" s="80"/>
+      <c r="G12" s="80"/>
+      <c r="H12" s="80"/>
+      <c r="I12" s="80"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
@@ -2202,17 +2202,17 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="55" t="s">
+      <c r="A21" s="87" t="s">
         <v>66</v>
       </c>
-      <c r="B21" s="55"/>
-      <c r="C21" s="55"/>
-      <c r="D21" s="55"/>
-      <c r="E21" s="55"/>
-      <c r="F21" s="55"/>
-      <c r="G21" s="55"/>
-      <c r="H21" s="55"/>
-      <c r="I21" s="55"/>
+      <c r="B21" s="87"/>
+      <c r="C21" s="87"/>
+      <c r="D21" s="87"/>
+      <c r="E21" s="87"/>
+      <c r="F21" s="87"/>
+      <c r="G21" s="87"/>
+      <c r="H21" s="87"/>
+      <c r="I21" s="87"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
@@ -2476,17 +2476,17 @@
       </c>
     </row>
     <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="58" t="s">
+      <c r="A32" s="88" t="s">
         <v>90</v>
       </c>
-      <c r="B32" s="58"/>
-      <c r="C32" s="58"/>
-      <c r="D32" s="58"/>
-      <c r="E32" s="58"/>
-      <c r="F32" s="58"/>
-      <c r="G32" s="58"/>
-      <c r="H32" s="58"/>
-      <c r="I32" s="58"/>
+      <c r="B32" s="88"/>
+      <c r="C32" s="88"/>
+      <c r="D32" s="88"/>
+      <c r="E32" s="88"/>
+      <c r="F32" s="88"/>
+      <c r="G32" s="88"/>
+      <c r="H32" s="88"/>
+      <c r="I32" s="88"/>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
@@ -2562,16 +2562,16 @@
       <c r="E36" s="48" t="s">
         <v>141</v>
       </c>
-      <c r="F36" s="90" t="s">
+      <c r="F36" s="75" t="s">
         <v>179</v>
       </c>
       <c r="G36" s="48" t="s">
         <v>160</v>
       </c>
-      <c r="H36" s="91" t="s">
+      <c r="H36" s="76" t="s">
         <v>106</v>
       </c>
-      <c r="I36" s="92" t="s">
+      <c r="I36" s="77" t="s">
         <v>159</v>
       </c>
       <c r="J36" s="45">
@@ -2583,17 +2583,12 @@
       <c r="L36" s="48">
         <v>7</v>
       </c>
-      <c r="M36" s="93">
+      <c r="M36" s="78">
         <v>2026</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B6:I6"/>
     <mergeCell ref="A21:I21"/>
     <mergeCell ref="A32:I32"/>
     <mergeCell ref="B7:I7"/>
@@ -2601,6 +2596,11 @@
     <mergeCell ref="B9:I9"/>
     <mergeCell ref="B10:I10"/>
     <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B6:I6"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I36" xr:uid="{1D3A478F-344B-4E54-B296-768D75F24C9F}">
@@ -2628,65 +2628,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="79" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
     </row>
     <row r="3" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="57"/>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
+      <c r="A3" s="86"/>
+      <c r="B3" s="86"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="86"/>
+      <c r="E3" s="86"/>
     </row>
     <row r="4" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="85" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
+      <c r="B4" s="85"/>
+      <c r="C4" s="85"/>
+      <c r="D4" s="85"/>
+      <c r="E4" s="85"/>
     </row>
     <row r="5" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="54" t="s">
+      <c r="A5" s="85" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
+      <c r="B5" s="85"/>
+      <c r="C5" s="85"/>
+      <c r="D5" s="85"/>
+      <c r="E5" s="85"/>
     </row>
     <row r="6" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="54" t="s">
+      <c r="A6" s="85" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="54"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
+      <c r="B6" s="85"/>
+      <c r="C6" s="85"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="85"/>
     </row>
     <row r="7" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="54" t="s">
+      <c r="A7" s="85" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="54"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
+      <c r="B7" s="85"/>
+      <c r="C7" s="85"/>
+      <c r="D7" s="85"/>
+      <c r="E7" s="85"/>
     </row>
     <row r="9" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="87" t="s">
+      <c r="A9" s="89" t="s">
         <v>114</v>
       </c>
-      <c r="B9" s="88"/>
-      <c r="C9" s="88"/>
-      <c r="D9" s="88"/>
-      <c r="E9" s="89"/>
+      <c r="B9" s="90"/>
+      <c r="C9" s="90"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="91"/>
     </row>
     <row r="10" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="37" t="s">
@@ -2757,476 +2757,479 @@
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="83" t="s">
+      <c r="A15" s="92" t="s">
         <v>113</v>
       </c>
-      <c r="B15" s="84"/>
-      <c r="C15" s="84"/>
-      <c r="D15" s="84"/>
-      <c r="E15" s="84"/>
-      <c r="F15" s="84"/>
-      <c r="G15" s="84"/>
+      <c r="B15" s="93"/>
+      <c r="C15" s="93"/>
+      <c r="D15" s="93"/>
+      <c r="E15" s="93"/>
+      <c r="F15" s="93"/>
+      <c r="G15" s="93"/>
     </row>
     <row r="16" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="62" t="s">
+      <c r="A16" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="62" t="s">
+      <c r="B16" s="54" t="s">
         <v>156</v>
       </c>
-      <c r="C16" s="63" t="s">
+      <c r="C16" s="55" t="s">
         <v>154</v>
       </c>
-      <c r="D16" s="62" t="s">
+      <c r="D16" s="54" t="s">
         <v>155</v>
       </c>
-      <c r="E16" s="62" t="s">
+      <c r="E16" s="54" t="s">
         <v>157</v>
       </c>
-      <c r="F16" s="64" t="s">
+      <c r="F16" s="56" t="s">
         <v>93</v>
       </c>
-      <c r="G16" s="64" t="s">
+      <c r="G16" s="56" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="65" t="s">
+      <c r="A17" s="57" t="s">
         <v>138</v>
       </c>
-      <c r="B17" s="67" t="s">
+      <c r="B17" s="59" t="s">
         <v>139</v>
       </c>
-      <c r="C17" s="66">
+      <c r="C17" s="58">
         <v>3500000</v>
       </c>
-      <c r="D17" s="68" t="s">
+      <c r="D17" s="60" t="s">
         <v>158</v>
       </c>
-      <c r="E17" s="69" t="s">
+      <c r="E17" s="61" t="s">
         <v>140</v>
       </c>
-      <c r="F17" s="70" t="s">
+      <c r="F17" s="62" t="s">
         <v>142</v>
       </c>
-      <c r="G17" s="70" t="s">
+      <c r="G17" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="67" t="s">
+      <c r="A18" s="59" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="71" t="s">
+      <c r="B18" s="63" t="s">
         <v>117</v>
       </c>
-      <c r="C18" s="66">
+      <c r="C18" s="58">
         <v>3000000</v>
       </c>
-      <c r="D18" s="67" t="s">
+      <c r="D18" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E18" s="72" t="s">
+      <c r="E18" s="64" t="s">
         <v>149</v>
       </c>
-      <c r="F18" s="70" t="s">
+      <c r="F18" s="62" t="s">
         <v>160</v>
       </c>
-      <c r="G18" s="70" t="s">
+      <c r="G18" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="67" t="s">
+      <c r="A19" s="59" t="s">
         <v>161</v>
       </c>
-      <c r="B19" s="71" t="s">
+      <c r="B19" s="63" t="s">
         <v>162</v>
       </c>
-      <c r="C19" s="66">
+      <c r="C19" s="58">
         <v>1950000</v>
       </c>
-      <c r="D19" s="67" t="s">
+      <c r="D19" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E19" s="73" t="s">
+      <c r="E19" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="F19" s="70" t="s">
+      <c r="F19" s="62" t="s">
         <v>163</v>
       </c>
-      <c r="G19" s="70" t="s">
+      <c r="G19" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="67" t="s">
+      <c r="A20" s="59" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="71" t="s">
+      <c r="B20" s="63" t="s">
         <v>102</v>
       </c>
-      <c r="C20" s="66">
+      <c r="C20" s="58">
         <v>1572931.74</v>
       </c>
-      <c r="D20" s="67" t="s">
+      <c r="D20" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E20" s="74" t="s">
+      <c r="E20" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="F20" s="75" t="s">
+      <c r="F20" s="67" t="s">
         <v>164</v>
       </c>
-      <c r="G20" s="70" t="s">
+      <c r="G20" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="67" t="s">
+      <c r="A21" s="59" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="71" t="s">
+      <c r="B21" s="63" t="s">
         <v>165</v>
       </c>
-      <c r="C21" s="66">
+      <c r="C21" s="58">
         <v>1100000</v>
       </c>
-      <c r="D21" s="67" t="s">
+      <c r="D21" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E21" s="73" t="s">
+      <c r="E21" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="F21" s="75" t="s">
+      <c r="F21" s="67" t="s">
         <v>164</v>
       </c>
-      <c r="G21" s="70" t="s">
+      <c r="G21" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="67" t="s">
+      <c r="A22" s="59" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="71" t="s">
+      <c r="B22" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="66">
+      <c r="C22" s="58">
         <v>1004484</v>
       </c>
-      <c r="D22" s="67" t="s">
+      <c r="D22" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E22" s="73" t="s">
+      <c r="E22" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="F22" s="76" t="s">
+      <c r="F22" s="68" t="s">
         <v>142</v>
       </c>
-      <c r="G22" s="70" t="s">
+      <c r="G22" s="62" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="67" t="s">
+      <c r="A23" s="59" t="s">
         <v>108</v>
       </c>
-      <c r="B23" s="71" t="s">
+      <c r="B23" s="63" t="s">
         <v>116</v>
       </c>
-      <c r="C23" s="66">
+      <c r="C23" s="58">
         <v>1000000</v>
       </c>
-      <c r="D23" s="67" t="s">
+      <c r="D23" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E23" s="72" t="s">
+      <c r="E23" s="64" t="s">
         <v>149</v>
       </c>
-      <c r="F23" s="70" t="s">
+      <c r="F23" s="62" t="s">
         <v>163</v>
       </c>
-      <c r="G23" s="70" t="s">
+      <c r="G23" s="62" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="67" t="s">
+      <c r="A24" s="59" t="s">
         <v>166</v>
       </c>
-      <c r="B24" s="67" t="s">
+      <c r="B24" s="59" t="s">
         <v>167</v>
       </c>
-      <c r="C24" s="66">
+      <c r="C24" s="58">
         <v>840000</v>
       </c>
-      <c r="D24" s="67"/>
-      <c r="E24" s="69" t="s">
+      <c r="D24" s="59" t="s">
+        <v>158</v>
+      </c>
+      <c r="E24" s="61" t="s">
         <v>140</v>
       </c>
-      <c r="F24" s="75" t="s">
+      <c r="F24" s="67" t="s">
         <v>164</v>
       </c>
-      <c r="G24" s="70" t="s">
+      <c r="G24" s="62" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="67" t="s">
+      <c r="A25" s="59" t="s">
         <v>148</v>
       </c>
-      <c r="B25" s="71" t="s">
+      <c r="B25" s="63" t="s">
         <v>104</v>
       </c>
-      <c r="C25" s="66">
+      <c r="C25" s="58">
         <v>824838</v>
       </c>
-      <c r="D25" s="67" t="s">
+      <c r="D25" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E25" s="72" t="s">
+      <c r="E25" s="64" t="s">
         <v>149</v>
       </c>
-      <c r="F25" s="70" t="s">
+      <c r="F25" s="62" t="s">
         <v>142</v>
       </c>
-      <c r="G25" s="70" t="s">
+      <c r="G25" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="67" t="s">
+      <c r="A26" s="59" t="s">
         <v>168</v>
       </c>
-      <c r="B26" s="71" t="s">
+      <c r="B26" s="63" t="s">
         <v>103</v>
       </c>
-      <c r="C26" s="66">
+      <c r="C26" s="58">
         <v>620035.83999999997</v>
       </c>
-      <c r="D26" s="67" t="s">
+      <c r="D26" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E26" s="69" t="s">
+      <c r="E26" s="61" t="s">
         <v>140</v>
       </c>
-      <c r="F26" s="75" t="s">
+      <c r="F26" s="67" t="s">
         <v>164</v>
       </c>
-      <c r="G26" s="70" t="s">
+      <c r="G26" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="67" t="s">
+      <c r="A27" s="59" t="s">
         <v>105</v>
       </c>
-      <c r="B27" s="71" t="s">
+      <c r="B27" s="63" t="s">
         <v>169</v>
       </c>
-      <c r="C27" s="66">
+      <c r="C27" s="58">
         <v>274409.84999999998</v>
       </c>
-      <c r="D27" s="67" t="s">
+      <c r="D27" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E27" s="72" t="s">
+      <c r="E27" s="64" t="s">
         <v>149</v>
       </c>
-      <c r="F27" s="70" t="s">
+      <c r="F27" s="62" t="s">
         <v>164</v>
       </c>
-      <c r="G27" s="70" t="s">
+      <c r="G27" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="67" t="s">
+      <c r="A28" s="59" t="s">
         <v>112</v>
       </c>
-      <c r="B28" s="71" t="s">
+      <c r="B28" s="63" t="s">
         <v>170</v>
       </c>
-      <c r="C28" s="66">
+      <c r="C28" s="58">
         <v>250000</v>
       </c>
-      <c r="D28" s="67" t="s">
+      <c r="D28" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E28" s="73" t="s">
+      <c r="E28" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="F28" s="76" t="s">
+      <c r="F28" s="68" t="s">
         <v>164</v>
       </c>
-      <c r="G28" s="70" t="s">
+      <c r="G28" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="67" t="s">
+      <c r="A29" s="59" t="s">
         <v>148</v>
       </c>
-      <c r="B29" s="71" t="s">
+      <c r="B29" s="63" t="s">
         <v>150</v>
       </c>
-      <c r="C29" s="66">
+      <c r="C29" s="58">
         <v>167000</v>
       </c>
-      <c r="D29" s="67" t="s">
+      <c r="D29" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E29" s="74" t="s">
+      <c r="E29" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="F29" s="70" t="s">
+      <c r="F29" s="62" t="s">
         <v>142</v>
       </c>
-      <c r="G29" s="70" t="s">
+      <c r="G29" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="67" t="s">
+      <c r="A30" s="59" t="s">
         <v>101</v>
       </c>
-      <c r="B30" s="71" t="s">
+      <c r="B30" s="63" t="s">
         <v>172</v>
       </c>
-      <c r="C30" s="66">
+      <c r="C30" s="58">
         <v>150000</v>
       </c>
-      <c r="D30" s="67" t="s">
+      <c r="D30" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E30" s="72" t="s">
+      <c r="E30" s="64" t="s">
         <v>149</v>
       </c>
-      <c r="F30" s="76" t="s">
+      <c r="F30" s="68" t="s">
         <v>164</v>
       </c>
-      <c r="G30" s="70" t="s">
+      <c r="G30" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="67" t="s">
+      <c r="A31" s="59" t="s">
         <v>110</v>
       </c>
-      <c r="B31" s="71" t="s">
+      <c r="B31" s="63" t="s">
         <v>111</v>
       </c>
-      <c r="C31" s="66">
+      <c r="C31" s="58">
         <v>128992.98</v>
       </c>
-      <c r="D31" s="67" t="s">
+      <c r="D31" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E31" s="69" t="s">
+      <c r="E31" s="61" t="s">
         <v>140</v>
       </c>
-      <c r="F31" s="76" t="s">
+      <c r="F31" s="68" t="s">
         <v>164</v>
       </c>
-      <c r="G31" s="70" t="s">
+      <c r="G31" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="67" t="s">
+      <c r="A32" s="59" t="s">
         <v>171</v>
       </c>
-      <c r="B32" s="71" t="s">
+      <c r="B32" s="63" t="s">
         <v>153</v>
       </c>
-      <c r="C32" s="66">
+      <c r="C32" s="58">
         <v>120000</v>
       </c>
-      <c r="D32" s="67" t="s">
+      <c r="D32" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E32" s="69" t="s">
+      <c r="E32" s="61" t="s">
         <v>140</v>
       </c>
-      <c r="F32" s="76" t="s">
+      <c r="F32" s="68" t="s">
         <v>163</v>
       </c>
-      <c r="G32" s="70" t="s">
+      <c r="G32" s="62" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="67" t="s">
+      <c r="A33" s="59" t="s">
         <v>173</v>
       </c>
-      <c r="B33" s="71" t="s">
+      <c r="B33" s="63" t="s">
         <v>174</v>
       </c>
-      <c r="C33" s="66">
+      <c r="C33" s="58">
         <v>100000</v>
       </c>
-      <c r="D33" s="67" t="s">
+      <c r="D33" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="E33" s="72" t="s">
+      <c r="E33" s="64" t="s">
         <v>149</v>
       </c>
-      <c r="F33" s="76" t="s">
+      <c r="F33" s="68" t="s">
         <v>164</v>
       </c>
-      <c r="G33" s="70" t="s">
+      <c r="G33" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="77" t="s">
+      <c r="A34" s="69" t="s">
         <v>109</v>
       </c>
-      <c r="B34" s="79" t="s">
+      <c r="B34" s="71" t="s">
         <v>175</v>
       </c>
-      <c r="C34" s="78">
+      <c r="C34" s="70">
         <v>35000</v>
       </c>
-      <c r="D34" s="77" t="s">
+      <c r="D34" s="69" t="s">
         <v>158</v>
       </c>
-      <c r="E34" s="80" t="s">
+      <c r="E34" s="72" t="s">
         <v>28</v>
       </c>
-      <c r="F34" s="70" t="s">
+      <c r="F34" s="62" t="s">
         <v>176</v>
       </c>
-      <c r="G34" s="70" t="s">
+      <c r="G34" s="62" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="77" t="s">
+      <c r="A35" s="69" t="s">
         <v>112</v>
       </c>
-      <c r="B35" s="79" t="s">
+      <c r="B35" s="71" t="s">
         <v>177</v>
       </c>
-      <c r="C35" s="78">
+      <c r="C35" s="70">
         <v>30600</v>
       </c>
-      <c r="D35" s="77" t="s">
+      <c r="D35" s="69" t="s">
         <v>158</v>
       </c>
-      <c r="E35" s="81" t="s">
+      <c r="E35" s="73" t="s">
         <v>43</v>
       </c>
-      <c r="F35" s="82" t="s">
+      <c r="F35" s="74" t="s">
         <v>178</v>
       </c>
-      <c r="G35" s="70" t="s">
+      <c r="G35" s="62" t="s">
         <v>141</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A15:G15"/>
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A1:E1"/>
@@ -3234,7 +3237,6 @@
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A15:G15"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E17:E35" xr:uid="{2EF9A1E0-747A-43D2-B879-3D0774406198}">
@@ -3256,17 +3258,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="79" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="79"/>
       <c r="J1" s="18"/>
       <c r="K1" s="18"/>
     </row>
@@ -3297,17 +3299,17 @@
       <c r="K3" s="18"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="80" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="60"/>
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="60"/>
-      <c r="H4" s="60"/>
-      <c r="I4" s="60"/>
+      <c r="B4" s="81"/>
+      <c r="C4" s="81"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="81"/>
+      <c r="I4" s="81"/>
       <c r="J4" s="18"/>
       <c r="K4" s="18"/>
     </row>
@@ -3364,16 +3366,16 @@
       <c r="K7" s="18"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="61" t="s">
+      <c r="A8" s="82" t="s">
         <v>114</v>
       </c>
-      <c r="B8" s="61"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
+      <c r="B8" s="82"/>
+      <c r="C8" s="82"/>
+      <c r="D8" s="82"/>
+      <c r="E8" s="82"/>
+      <c r="F8" s="82"/>
+      <c r="G8" s="82"/>
+      <c r="H8" s="82"/>
       <c r="I8" s="18"/>
       <c r="J8" s="18"/>
       <c r="K8" s="18"/>
@@ -3557,11 +3559,11 @@
       <c r="K15" s="30"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="85" t="s">
+      <c r="A16" s="83" t="s">
         <v>152</v>
       </c>
-      <c r="B16" s="86"/>
-      <c r="C16" s="86"/>
+      <c r="B16" s="84"/>
+      <c r="C16" s="84"/>
       <c r="J16" s="18"/>
       <c r="K16" s="18"/>
     </row>

</xml_diff>